<commit_message>
update with new average - start
</commit_message>
<xml_diff>
--- a/Data/Copy of Data Linking figure extract - AEMO meter data.xlsx
+++ b/Data/Copy of Data Linking figure extract - AEMO meter data.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{21CCCFFC-F38B-4302-802D-E9B1FCCAF537}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="5" xr2:uid="{5E18ABAC-37F5-4270-BC2D-91396A011EC6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{5E18ABAC-37F5-4270-BC2D-91396A011EC6}"/>
   </bookViews>
   <sheets>
     <sheet name="Figure 5" sheetId="20" r:id="rId1"/>
@@ -16988,15 +16988,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_dlc_DocId xmlns="a14523ce-dede-483e-883a-2d83261080bd">NETWORKDEV-489286805-319</_dlc_DocId>
-    <_dlc_DocIdUrl xmlns="a14523ce-dede-483e-883a-2d83261080bd">
-      <Url>http://sharedocs/sites/nd/BusinessAsUsual/_layouts/15/DocIdRedir.aspx?ID=NETWORKDEV-489286805-319</Url>
-      <Description>NETWORKDEV-489286805-319</Description>
-    </_dlc_DocIdUrl>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -17145,12 +17142,15 @@
 </file>
 
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_dlc_DocId xmlns="a14523ce-dede-483e-883a-2d83261080bd">NETWORKDEV-489286805-319</_dlc_DocId>
+    <_dlc_DocIdUrl xmlns="a14523ce-dede-483e-883a-2d83261080bd">
+      <Url>http://sharedocs/sites/nd/BusinessAsUsual/_layouts/15/DocIdRedir.aspx?ID=NETWORKDEV-489286805-319</Url>
+      <Description>NETWORKDEV-489286805-319</Description>
+    </_dlc_DocIdUrl>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -17162,17 +17162,9 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BEB7703D-23C5-427C-AF59-13D3B9C39B0E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B20DBDEF-43A6-4B1D-85FE-78297E03FAAE}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="a14523ce-dede-483e-883a-2d83261080bd"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -17196,9 +17188,17 @@
 </file>
 
 <file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B20DBDEF-43A6-4B1D-85FE-78297E03FAAE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BEB7703D-23C5-427C-AF59-13D3B9C39B0E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a14523ce-dede-483e-883a-2d83261080bd"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>